<commit_message>
Bảng phân công công việc
Phân công lại đầy đủ hơn.
</commit_message>
<xml_diff>
--- a/Bảng phân công công việc nhóm 7.xlsx
+++ b/Bảng phân công công việc nhóm 7.xlsx
@@ -56,7 +56,7 @@
     <t>083306010188</t>
   </si>
   <si>
-    <t>Slide, Doc, Giao diện màn hình chính (Slidebar+Khung chat)</t>
+    <t>Slide, Giao diện màn hình chính (Slidebar+Khung chat)</t>
   </si>
   <si>
     <t>Đỗ Hoàng Hải</t>
@@ -74,7 +74,7 @@
     <t>079306005139</t>
   </si>
   <si>
-    <t>Slide, Doc, Giao diện bảng chọn emoji</t>
+    <t>Slide, Giao diện bảng chọn emoji</t>
   </si>
   <si>
     <t>Phạm Minh Phúc</t>
@@ -83,7 +83,7 @@
     <t>077206000235</t>
   </si>
   <si>
-    <t>Slide, Doc, Giao diện bong bóng chat</t>
+    <t>Slide, Giao diện bong bóng chat</t>
   </si>
   <si>
     <t>Đoàn Trần Nhật Vy</t>

</xml_diff>